<commit_message>
feat: add modified date tracking to Bosch and Lucas stock import processes, update models and frontend display
</commit_message>
<xml_diff>
--- a/backend/public/BOSCH_STOCK1.xlsx
+++ b/backend/public/BOSCH_STOCK1.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abc\Desktop\bk eng stock\updateStock\Update-Stock\backend\public\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A584694-3E3E-41C7-B574-736F127BD8DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="15600" windowHeight="11160" tabRatio="730" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="12240" windowHeight="9240" tabRatio="730"/>
   </bookViews>
   <sheets>
     <sheet name="ELEMENT" sheetId="1" r:id="rId1"/>
@@ -48,7 +42,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="5">'DIESEL FILTER&amp;OIL FILTER'!$A$3:$N$634</definedName>
     <definedName name="Z_8145F22A_AD74_4799_898B_BCECC4FA34F9_.wvu.PrintArea" localSheetId="5" hidden="1">'DIESEL FILTER&amp;OIL FILTER'!$A$3:$N$634</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="124519"/>
   <customWorkbookViews>
     <customWorkbookView name="pcs - Personal View" guid="{8145F22A-AD74-4799-898B-BCECC4FA34F9}" mergeInterval="0" personalView="1" maximized="1" xWindow="1" yWindow="1" windowWidth="800" windowHeight="379" tabRatio="628" activeSheetId="5"/>
   </customWorkbookViews>
@@ -10940,10 +10934,10 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
+    <numFmt numFmtId="44" formatCode="_ &quot;Rs.&quot;\ * #,##0.00_ ;_ &quot;Rs.&quot;\ * \-#,##0.00_ ;_ &quot;Rs.&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="164" formatCode="_ &quot;Rs.&quot;\ * #,##0.00_ ;_ &quot;Rs.&quot;\ * \-#,##0.00_ ;_ &quot;Rs.&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="34">
     <font>
@@ -11253,7 +11247,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
@@ -11464,7 +11458,7 @@
     <xf numFmtId="0" fontId="28" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="20" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -11507,10 +11501,10 @@
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="4" builtinId="3"/>
-    <cellStyle name="Comma 2" xfId="5" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Comma 2" xfId="5"/>
     <cellStyle name="Currency" xfId="3" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 3" xfId="2" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="Normal 3" xfId="2"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="32">
@@ -11912,9 +11906,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -11952,7 +11946,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -11986,7 +11980,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -12021,10 +12014,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -12197,7 +12189,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:J440"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
@@ -13593,7 +13585,7 @@
       </c>
       <c r="D66" s="17"/>
       <c r="E66" s="19">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F66" s="17"/>
       <c r="G66" s="17"/>
@@ -13909,7 +13901,7 @@
       </c>
       <c r="D82" s="17"/>
       <c r="E82" s="19">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F82" s="17"/>
       <c r="G82" s="17"/>
@@ -13928,7 +13920,7 @@
       </c>
       <c r="D83" s="17"/>
       <c r="E83" s="19">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F83" s="17"/>
       <c r="G83" s="17"/>
@@ -15047,7 +15039,7 @@
       </c>
       <c r="D136" s="17"/>
       <c r="E136" s="19">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F136" s="17"/>
       <c r="G136" s="17"/>
@@ -15672,7 +15664,7 @@
         <v>2168</v>
       </c>
       <c r="E167" s="19">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F167" s="17" t="s">
         <v>2167</v>
@@ -16085,7 +16077,8 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F172" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <sheetProtection password="CF21" sheet="1" objects="1" scenarios="1"/>
+  <autoFilter ref="A1:F172"/>
   <customSheetViews>
     <customSheetView guid="{8145F22A-AD74-4799-898B-BCECC4FA34F9}" scale="110" topLeftCell="A104">
       <selection activeCell="G107" sqref="G107"/>
@@ -16099,7 +16092,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet10"/>
   <dimension ref="A1:H293"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -16170,7 +16163,7 @@
         <v>1826</v>
       </c>
       <c r="E3" s="75">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F3" s="74">
         <v>1974</v>
@@ -17506,7 +17499,7 @@
         <v>387</v>
       </c>
       <c r="E72" s="75">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F72" s="74">
         <v>2206</v>
@@ -18762,7 +18755,7 @@
         <v>2076</v>
       </c>
       <c r="E137" s="75">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F137" s="74" t="s">
         <v>2793</v>
@@ -18862,7 +18855,7 @@
         <v>822</v>
       </c>
       <c r="E142" s="75">
-        <v>79</v>
+        <v>128</v>
       </c>
       <c r="F142" s="74">
         <v>746</v>
@@ -19532,7 +19525,7 @@
         <v>2704</v>
       </c>
       <c r="E175" s="75">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F175" s="74">
         <v>1947</v>
@@ -20114,7 +20107,7 @@
       </c>
       <c r="D204" s="74"/>
       <c r="E204" s="75">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F204" s="74">
         <v>2434</v>
@@ -20534,7 +20527,7 @@
         <v>1859</v>
       </c>
       <c r="E225" s="75">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F225" s="74">
         <v>9251</v>
@@ -20622,7 +20615,7 @@
         <v>2443</v>
       </c>
       <c r="E229" s="75">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F229" s="74">
         <v>12762</v>
@@ -21872,7 +21865,7 @@
       </c>
       <c r="D287" s="74"/>
       <c r="E287" s="75">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F287" s="74">
         <v>10302</v>
@@ -21998,7 +21991,7 @@
     </row>
   </sheetData>
   <sheetProtection password="CF21" sheet="1" objects="1" scenarios="1"/>
-  <autoFilter ref="A1:I293" xr:uid="{00000000-0009-0000-0000-000009000000}"/>
+  <autoFilter ref="A1:I293"/>
   <customSheetViews>
     <customSheetView guid="{8145F22A-AD74-4799-898B-BCECC4FA34F9}" scale="110" topLeftCell="A1208">
       <selection activeCell="D1139" sqref="D1139"/>
@@ -22043,7 +22036,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet11"/>
   <dimension ref="A1:H1391"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -22133,7 +22126,7 @@
         <v>3508</v>
       </c>
       <c r="E4" s="71">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="F4" s="70">
         <v>287</v>
@@ -22155,7 +22148,7 @@
         <v>3509</v>
       </c>
       <c r="E5" s="71">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="F5" s="70">
         <v>167</v>
@@ -22177,7 +22170,7 @@
         <v>3510</v>
       </c>
       <c r="E6" s="71">
-        <v>141</v>
+        <v>121</v>
       </c>
       <c r="F6" s="70">
         <v>182</v>
@@ -31175,7 +31168,7 @@
     </row>
   </sheetData>
   <sheetProtection password="CF21" sheet="1" objects="1" scenarios="1"/>
-  <autoFilter ref="A1:H54" xr:uid="{00000000-0009-0000-0000-00000A000000}"/>
+  <autoFilter ref="A1:H54"/>
   <customSheetViews>
     <customSheetView guid="{8145F22A-AD74-4799-898B-BCECC4FA34F9}" scale="120" topLeftCell="A52">
       <selection activeCell="D57" sqref="D57"/>
@@ -31196,7 +31189,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet12"/>
   <dimension ref="A1:H311"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12"/>
@@ -31286,7 +31279,7 @@
         <v>1295</v>
       </c>
       <c r="E4" s="19">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F4" s="17">
         <v>1772</v>
@@ -31870,7 +31863,7 @@
         <v>2374</v>
       </c>
       <c r="E32" s="19">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="F32" s="17">
         <v>2740</v>
@@ -32120,7 +32113,7 @@
         <v>1331</v>
       </c>
       <c r="E44" s="19">
-        <v>449</v>
+        <v>389</v>
       </c>
       <c r="F44" s="17">
         <v>247</v>
@@ -32141,7 +32134,7 @@
         <v>1331</v>
       </c>
       <c r="E45" s="19">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="F45" s="17">
         <v>676</v>
@@ -32505,7 +32498,7 @@
       </c>
       <c r="D63" s="32"/>
       <c r="E63" s="84">
-        <v>220</v>
+        <v>140</v>
       </c>
       <c r="F63" s="32">
         <v>115</v>
@@ -33092,7 +33085,7 @@
     </row>
   </sheetData>
   <sheetProtection password="CF21" sheet="1" objects="1" scenarios="1"/>
-  <autoFilter ref="A1:H92" xr:uid="{00000000-0009-0000-0000-00000B000000}"/>
+  <autoFilter ref="A1:H92"/>
   <customSheetViews>
     <customSheetView guid="{8145F22A-AD74-4799-898B-BCECC4FA34F9}" scale="115" topLeftCell="A35">
       <selection activeCell="D44" sqref="D44"/>
@@ -33109,7 +33102,7 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet19"/>
   <dimension ref="A1:F99"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -33935,7 +33928,7 @@
         <v>2506</v>
       </c>
       <c r="E41">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F41">
         <v>561</v>
@@ -35026,7 +35019,7 @@
     </row>
   </sheetData>
   <sheetProtection password="CF21" sheet="1" objects="1" scenarios="1"/>
-  <autoFilter ref="A1:F98" xr:uid="{00000000-0009-0000-0000-00000C000000}"/>
+  <autoFilter ref="A1:F98"/>
   <customSheetViews>
     <customSheetView guid="{8145F22A-AD74-4799-898B-BCECC4FA34F9}">
       <selection activeCell="A2" sqref="A2"/>
@@ -35042,7 +35035,7 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet13"/>
   <dimension ref="A2:C18"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -35123,7 +35116,7 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet14"/>
   <dimension ref="A1:K50"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -35714,7 +35707,7 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet18"/>
   <dimension ref="A3:I20"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -35887,7 +35880,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet2">
     <tabColor rgb="FF00B0F0"/>
   </sheetPr>
@@ -36578,7 +36571,7 @@
       </c>
       <c r="D38" s="26"/>
       <c r="E38" s="10">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F38" s="9"/>
     </row>
@@ -41303,7 +41296,7 @@
     </row>
   </sheetData>
   <sheetProtection password="CF21" sheet="1" objects="1" scenarios="1"/>
-  <autoFilter ref="A1:G275" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:G275"/>
   <customSheetViews>
     <customSheetView guid="{8145F22A-AD74-4799-898B-BCECC4FA34F9}" topLeftCell="A335">
       <selection activeCell="C348" sqref="C348"/>
@@ -41317,7 +41310,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:H772"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -44970,7 +44963,7 @@
     </row>
   </sheetData>
   <sheetProtection password="CF21" sheet="1" objects="1" scenarios="1"/>
-  <autoFilter ref="A1:H129" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <autoFilter ref="A1:H129"/>
   <customSheetViews>
     <customSheetView guid="{8145F22A-AD74-4799-898B-BCECC4FA34F9}" scale="110" topLeftCell="A239">
       <selection activeCell="D241" sqref="D241"/>
@@ -44984,7 +44977,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:H478"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -45118,7 +45111,7 @@
       </c>
       <c r="D7" s="33"/>
       <c r="E7" s="35">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F7" s="33">
         <v>502</v>
@@ -46365,7 +46358,7 @@
       </c>
       <c r="D84" s="33"/>
       <c r="E84" s="35">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F84" s="33"/>
     </row>
@@ -47146,7 +47139,7 @@
       </c>
       <c r="D132" s="33"/>
       <c r="E132" s="35">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F132" s="33">
         <v>247</v>
@@ -49225,7 +49218,7 @@
       </c>
       <c r="D257" s="33"/>
       <c r="E257" s="35">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="F257" s="33">
         <v>137</v>
@@ -49261,7 +49254,7 @@
         <v>2724</v>
       </c>
       <c r="E259" s="35">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F259" s="33">
         <v>327</v>
@@ -49739,7 +49732,7 @@
       </c>
       <c r="D288" s="33"/>
       <c r="E288" s="35">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="F288" s="33"/>
     </row>
@@ -49863,7 +49856,7 @@
       </c>
       <c r="D295" s="33"/>
       <c r="E295" s="35">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F295" s="33">
         <v>696</v>
@@ -50226,7 +50219,7 @@
       </c>
       <c r="D316" s="33"/>
       <c r="E316" s="35">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F316" s="33">
         <v>865</v>
@@ -50334,7 +50327,7 @@
         <v>3591</v>
       </c>
       <c r="E322" s="35">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F322" s="33" t="s">
         <v>2935</v>
@@ -50632,7 +50625,7 @@
         <v>3327</v>
       </c>
       <c r="E338" s="35">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F338" s="33">
         <v>9850</v>
@@ -50738,7 +50731,7 @@
         <v>3330</v>
       </c>
       <c r="E344" s="35">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F344" s="33">
         <v>6480</v>
@@ -51432,7 +51425,7 @@
     </row>
   </sheetData>
   <sheetProtection password="CF21" sheet="1" objects="1" scenarios="1"/>
-  <autoFilter ref="A1:H376" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
+  <autoFilter ref="A1:H376"/>
   <customSheetViews>
     <customSheetView guid="{8145F22A-AD74-4799-898B-BCECC4FA34F9}" scale="110" topLeftCell="A2437">
       <selection activeCell="D2444" sqref="D2444"/>
@@ -51446,7 +51439,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:G571"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -51761,7 +51754,7 @@
       </c>
       <c r="D19" s="33"/>
       <c r="E19" s="56">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F19" s="35">
         <v>2025</v>
@@ -51860,7 +51853,7 @@
         <v>2698</v>
       </c>
       <c r="E24" s="56">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="F24" s="35" t="s">
         <v>2820</v>
@@ -53019,7 +53012,7 @@
         <v>2708</v>
       </c>
       <c r="E91" s="56">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="F91" s="35">
         <v>855</v>
@@ -53145,7 +53138,7 @@
         <v>2704</v>
       </c>
       <c r="E98" s="56">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="F98" s="56">
         <v>1320</v>
@@ -53763,7 +53756,7 @@
         <v>2707</v>
       </c>
       <c r="E133" s="56">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F133" s="35" t="s">
         <v>3585</v>
@@ -53826,7 +53819,7 @@
         <v>518894</v>
       </c>
       <c r="E136" s="56">
-        <v>66</v>
+        <v>81</v>
       </c>
       <c r="F136" s="35" t="s">
         <v>3583</v>
@@ -54025,7 +54018,7 @@
         <v>2700</v>
       </c>
       <c r="E147" s="56">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F147" s="35">
         <v>554</v>
@@ -54085,7 +54078,7 @@
         <v>2703</v>
       </c>
       <c r="E150" s="56">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="F150" s="35">
         <v>893</v>
@@ -54552,7 +54545,7 @@
         <v>2704</v>
       </c>
       <c r="E175" s="56">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F175" s="56">
         <v>2310</v>
@@ -54630,7 +54623,7 @@
         <v>2704</v>
       </c>
       <c r="E179" s="56">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F179" s="35">
         <v>681</v>
@@ -54939,7 +54932,7 @@
         <v>2704</v>
       </c>
       <c r="E195" s="56">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F195" s="35">
         <v>4839</v>
@@ -55035,7 +55028,7 @@
         <v>2698</v>
       </c>
       <c r="E200" s="56">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="F200" s="35">
         <v>1399</v>
@@ -55123,7 +55116,7 @@
         <v>2704</v>
       </c>
       <c r="E205" s="56">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F205" s="35">
         <v>1199</v>
@@ -55518,7 +55511,7 @@
       </c>
       <c r="D227" s="33"/>
       <c r="E227" s="56">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F227" s="35">
         <v>2749</v>
@@ -57098,7 +57091,7 @@
     </row>
   </sheetData>
   <sheetProtection password="CF21" sheet="1" objects="1" scenarios="1"/>
-  <autoFilter ref="A1:G231" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
+  <autoFilter ref="A1:G231"/>
   <customSheetViews>
     <customSheetView guid="{8145F22A-AD74-4799-898B-BCECC4FA34F9}" scale="110" topLeftCell="A1207">
       <selection activeCell="F1213" sqref="F1213"/>
@@ -57124,7 +57117,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet6"/>
   <dimension ref="A1:J293"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -57184,7 +57177,7 @@
       </c>
       <c r="D3" s="33"/>
       <c r="E3" s="33">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F3" s="35">
         <v>161</v>
@@ -57202,7 +57195,7 @@
       </c>
       <c r="D4" s="33"/>
       <c r="E4" s="33">
-        <v>133</v>
+        <v>113</v>
       </c>
       <c r="F4" s="35">
         <v>146</v>
@@ -57309,7 +57302,7 @@
       </c>
       <c r="D10" s="33"/>
       <c r="E10" s="33">
-        <v>643</v>
+        <v>863</v>
       </c>
       <c r="F10" s="35">
         <v>193</v>
@@ -57327,7 +57320,7 @@
       </c>
       <c r="D11" s="33"/>
       <c r="E11" s="33">
-        <v>52</v>
+        <v>112</v>
       </c>
       <c r="F11" s="35">
         <v>184</v>
@@ -57345,7 +57338,7 @@
       </c>
       <c r="D12" s="33"/>
       <c r="E12" s="33">
-        <v>742</v>
+        <v>724</v>
       </c>
       <c r="F12" s="35">
         <v>184</v>
@@ -57422,7 +57415,7 @@
       </c>
       <c r="D16" s="33"/>
       <c r="E16" s="33">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="F16" s="35">
         <v>400</v>
@@ -57440,7 +57433,7 @@
       </c>
       <c r="D17" s="33"/>
       <c r="E17" s="33">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F17" s="35">
         <v>396</v>
@@ -57476,7 +57469,7 @@
       </c>
       <c r="D19" s="33"/>
       <c r="E19" s="33">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="F19" s="35" t="s">
         <v>2789</v>
@@ -57532,7 +57525,7 @@
       </c>
       <c r="D22" s="33"/>
       <c r="E22" s="33">
-        <v>312</v>
+        <v>305</v>
       </c>
       <c r="F22" s="35">
         <v>363</v>
@@ -57676,7 +57669,7 @@
         <v>3357</v>
       </c>
       <c r="E30" s="60">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="F30" s="33">
         <v>586</v>
@@ -57754,7 +57747,7 @@
       </c>
       <c r="D34" s="33"/>
       <c r="E34" s="53">
-        <v>138</v>
+        <v>121</v>
       </c>
       <c r="F34" s="35">
         <v>392</v>
@@ -57852,10 +57845,10 @@
       </c>
       <c r="D39" s="33"/>
       <c r="E39" s="33">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F39" s="35">
-        <v>2208</v>
+        <v>2318</v>
       </c>
     </row>
     <row r="40" spans="1:6">
@@ -57980,7 +57973,7 @@
         <v>3368</v>
       </c>
       <c r="E46" s="60">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="F46" s="35">
         <v>208</v>
@@ -58114,7 +58107,7 @@
         <v>3372</v>
       </c>
       <c r="E54" s="42">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F54" s="35">
         <v>211</v>
@@ -58150,7 +58143,7 @@
       </c>
       <c r="D56" s="33"/>
       <c r="E56" s="33">
-        <v>168</v>
+        <v>148</v>
       </c>
       <c r="F56" s="35">
         <v>120</v>
@@ -58168,7 +58161,7 @@
       </c>
       <c r="D57" s="33"/>
       <c r="E57" s="33">
-        <v>168</v>
+        <v>143</v>
       </c>
       <c r="F57" s="35">
         <v>260</v>
@@ -58256,7 +58249,7 @@
       </c>
       <c r="D62" s="33"/>
       <c r="E62" s="33">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="F62" s="35">
         <v>298</v>
@@ -58440,7 +58433,7 @@
       </c>
       <c r="D73" s="33"/>
       <c r="E73" s="42">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="F73" s="35">
         <v>295</v>
@@ -58498,7 +58491,7 @@
       </c>
       <c r="D76" s="33"/>
       <c r="E76" s="33">
-        <v>140</v>
+        <v>106</v>
       </c>
       <c r="F76" s="35">
         <v>239</v>
@@ -58516,7 +58509,7 @@
       </c>
       <c r="D77" s="33"/>
       <c r="E77" s="42">
-        <v>121</v>
+        <v>104</v>
       </c>
       <c r="F77" s="35">
         <v>124</v>
@@ -58534,7 +58527,7 @@
       </c>
       <c r="D78" s="33"/>
       <c r="E78" s="33">
-        <v>106</v>
+        <v>81</v>
       </c>
       <c r="F78" s="35">
         <v>253</v>
@@ -58677,7 +58670,9 @@
       <c r="D86" s="33" t="s">
         <v>3380</v>
       </c>
-      <c r="E86" s="33"/>
+      <c r="E86" s="33">
+        <v>5</v>
+      </c>
       <c r="F86" s="35">
         <v>410</v>
       </c>
@@ -58696,7 +58691,7 @@
         <v>3382</v>
       </c>
       <c r="E87" s="33">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F87" s="33">
         <v>330</v>
@@ -58802,7 +58797,7 @@
       </c>
       <c r="D93" s="33"/>
       <c r="E93" s="33">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F93" s="35">
         <v>1656</v>
@@ -58859,7 +58854,7 @@
       </c>
       <c r="D96" s="33"/>
       <c r="E96" s="33">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F96" s="35">
         <v>288</v>
@@ -59049,7 +59044,7 @@
         <v>3387</v>
       </c>
       <c r="E106" s="60">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="F106" s="35">
         <v>396</v>
@@ -59127,7 +59122,7 @@
         <v>1573</v>
       </c>
       <c r="E110" s="33">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="F110" s="35">
         <v>494</v>
@@ -59177,7 +59172,7 @@
       </c>
       <c r="D113" s="33"/>
       <c r="E113" s="33">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F113" s="35">
         <v>746</v>
@@ -59738,7 +59733,7 @@
         <v>1859</v>
       </c>
       <c r="E143" s="35">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F143" s="33">
         <v>371</v>
@@ -60029,7 +60024,7 @@
         <v>1859</v>
       </c>
       <c r="E160" s="33">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="F160" s="35">
         <v>234</v>
@@ -60049,7 +60044,7 @@
         <v>2423</v>
       </c>
       <c r="E161" s="33">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="F161" s="35">
         <v>300</v>
@@ -60089,7 +60084,7 @@
         <v>3409</v>
       </c>
       <c r="E163" s="33">
-        <v>59</v>
+        <v>124</v>
       </c>
       <c r="F163" s="35">
         <v>686</v>
@@ -60169,7 +60164,7 @@
         <v>2553</v>
       </c>
       <c r="E167" s="33">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F167" s="35" t="s">
         <v>2936</v>
@@ -60269,7 +60264,7 @@
         <v>3421</v>
       </c>
       <c r="E172" s="33">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="F172" s="35">
         <v>649</v>
@@ -60289,7 +60284,7 @@
         <v>3422</v>
       </c>
       <c r="E173" s="33">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="F173" s="35">
         <v>759</v>
@@ -60389,7 +60384,7 @@
         <v>3428</v>
       </c>
       <c r="E178" s="33">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="F178" s="35">
         <v>288</v>
@@ -60479,7 +60474,7 @@
         <v>290</v>
       </c>
       <c r="E183" s="33">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F183" s="35">
         <v>170</v>
@@ -60499,7 +60494,7 @@
         <v>318</v>
       </c>
       <c r="E184" s="33">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F184" s="35">
         <v>186</v>
@@ -60579,7 +60574,7 @@
         <v>2247</v>
       </c>
       <c r="E188" s="33">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F188" s="35">
         <v>229</v>
@@ -60599,7 +60594,7 @@
         <v>3433</v>
       </c>
       <c r="E189" s="33">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F189" s="35" t="s">
         <v>2788</v>
@@ -60619,7 +60614,7 @@
         <v>3434</v>
       </c>
       <c r="E190" s="33">
-        <v>75</v>
+        <v>119</v>
       </c>
       <c r="F190" s="33" t="s">
         <v>3023</v>
@@ -60815,7 +60810,7 @@
         <v>3440</v>
       </c>
       <c r="E200" s="33">
-        <v>71</v>
+        <v>147</v>
       </c>
       <c r="F200" s="35">
         <v>155</v>
@@ -61013,7 +61008,7 @@
         <v>3447</v>
       </c>
       <c r="E210" s="33">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="F210" s="35">
         <v>345</v>
@@ -61063,7 +61058,7 @@
         <v>836</v>
       </c>
       <c r="E213" s="33">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F213" s="35">
         <v>592</v>
@@ -61163,7 +61158,7 @@
         <v>3453</v>
       </c>
       <c r="E218" s="33">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F218" s="33" t="s">
         <v>2941</v>
@@ -61183,7 +61178,7 @@
         <v>2393</v>
       </c>
       <c r="E219" s="33">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F219" s="33">
         <v>244</v>
@@ -61323,7 +61318,7 @@
         <v>3459</v>
       </c>
       <c r="E226" s="33">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F226" s="33">
         <v>440</v>
@@ -61463,7 +61458,7 @@
         <v>3466</v>
       </c>
       <c r="E233" s="33">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F233" s="35">
         <v>353</v>
@@ -61941,7 +61936,7 @@
         <v>3067</v>
       </c>
       <c r="E257" s="33">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="F257" s="35">
         <v>546</v>
@@ -62019,7 +62014,7 @@
         <v>3066</v>
       </c>
       <c r="E261" s="33">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F261" s="35">
         <v>550</v>
@@ -62640,7 +62635,7 @@
     </row>
   </sheetData>
   <sheetProtection password="CF21" sheet="1" objects="1" scenarios="1"/>
-  <autoFilter ref="A1:J293" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
+  <autoFilter ref="A1:J293"/>
   <customSheetViews>
     <customSheetView guid="{8145F22A-AD74-4799-898B-BCECC4FA34F9}" scale="110" topLeftCell="A1045">
       <selection activeCell="D1055" sqref="D1055"/>
@@ -62664,7 +62659,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet7"/>
   <dimension ref="A1:H94"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -63787,7 +63782,7 @@
         <v>344</v>
       </c>
       <c r="E61" s="62">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F61" s="4">
         <v>2214</v>
@@ -64185,7 +64180,7 @@
     </row>
   </sheetData>
   <sheetProtection password="CF21" sheet="1" objects="1" scenarios="1"/>
-  <autoFilter ref="A1:F80" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
+  <autoFilter ref="A1:F80"/>
   <customSheetViews>
     <customSheetView guid="{8145F22A-AD74-4799-898B-BCECC4FA34F9}" scale="110" topLeftCell="A503">
       <selection activeCell="E514" sqref="E514"/>
@@ -64198,7 +64193,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet8"/>
   <dimension ref="A1:F43"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -64264,7 +64259,7 @@
         <v>290</v>
       </c>
       <c r="E3" s="35">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F3" s="33">
         <v>1465</v>
@@ -64993,8 +64988,8 @@
       <c r="F43" s="33"/>
     </row>
   </sheetData>
-  <sheetProtection password="CF21" sheet="1" objects="1" scenarios="1"/>
-  <autoFilter ref="A1:F43" xr:uid="{00000000-0009-0000-0000-000007000000}"/>
+  <sheetProtection password="CFE1" sheet="1" objects="1" scenarios="1"/>
+  <autoFilter ref="A1:F43"/>
   <customSheetViews>
     <customSheetView guid="{8145F22A-AD74-4799-898B-BCECC4FA34F9}" scale="120" topLeftCell="A217">
       <selection activeCell="C224" sqref="C224"/>
@@ -65007,7 +65002,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Sheet9"/>
   <dimension ref="A1:G119"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -65174,7 +65169,7 @@
       </c>
       <c r="D9" s="33"/>
       <c r="E9" s="35">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="F9" s="33" t="s">
         <v>2815</v>
@@ -65474,7 +65469,7 @@
       </c>
       <c r="D26" s="33"/>
       <c r="E26" s="35">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="F26" s="33">
         <v>18</v>
@@ -65524,7 +65519,7 @@
       </c>
       <c r="D29" s="33"/>
       <c r="E29" s="35">
-        <v>360</v>
+        <v>330</v>
       </c>
       <c r="F29" s="33">
         <v>21</v>
@@ -65953,7 +65948,7 @@
         <v>2290</v>
       </c>
       <c r="E53" s="35">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F53" s="33">
         <v>5355</v>
@@ -65973,7 +65968,7 @@
         <v>2295</v>
       </c>
       <c r="E54" s="35">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F54" s="33">
         <v>5355</v>
@@ -66015,7 +66010,7 @@
         <v>2670</v>
       </c>
       <c r="E57" s="35">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="F57" s="33">
         <v>750</v>
@@ -67013,7 +67008,7 @@
     </row>
   </sheetData>
   <sheetProtection password="CF21" sheet="1" objects="1" scenarios="1"/>
-  <autoFilter ref="A1:G119" xr:uid="{00000000-0009-0000-0000-000008000000}"/>
+  <autoFilter ref="A1:G119"/>
   <customSheetViews>
     <customSheetView guid="{8145F22A-AD74-4799-898B-BCECC4FA34F9}" scale="116" topLeftCell="A1179">
       <selection activeCell="F1188" sqref="F1188"/>

</xml_diff>

<commit_message>
feat: Add Bosch Price Detail page and update related components for improved navigation and data retrieval
</commit_message>
<xml_diff>
--- a/backend/public/BOSCH_STOCK1.xlsx
+++ b/backend/public/BOSCH_STOCK1.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="12240" windowHeight="9240" tabRatio="730"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="12240" windowHeight="9240" tabRatio="730" firstSheet="3" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="ELEMENT" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,6 @@
   <customWorkbookViews>
     <customWorkbookView name="pcs - Personal View" guid="{8145F22A-AD74-4799-898B-BCECC4FA34F9}" mergeInterval="0" personalView="1" maximized="1" xWindow="1" yWindow="1" windowWidth="800" windowHeight="379" tabRatio="628" activeSheetId="5"/>
   </customWorkbookViews>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -14277,7 +14276,7 @@
       </c>
       <c r="D100" s="17"/>
       <c r="E100" s="19">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F100" s="17" t="s">
         <v>2650</v>
@@ -16161,7 +16160,7 @@
         <v>1825</v>
       </c>
       <c r="E3" s="75">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="F3" s="74">
         <v>1974</v>
@@ -16415,7 +16414,7 @@
         <v>2703</v>
       </c>
       <c r="E15" s="75">
-        <v>22</v>
+        <v>82</v>
       </c>
       <c r="F15" s="74">
         <v>179</v>
@@ -17497,7 +17496,7 @@
         <v>387</v>
       </c>
       <c r="E72" s="75">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="F72" s="74">
         <v>2206</v>
@@ -19817,7 +19816,7 @@
       </c>
       <c r="D189" s="74"/>
       <c r="E189" s="75">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F189" s="74" t="s">
         <v>3580</v>
@@ -22043,7 +22042,7 @@
     <col min="2" max="2" width="37.85546875" customWidth="1"/>
     <col min="3" max="3" width="20.28515625" customWidth="1"/>
     <col min="4" max="4" width="22.7109375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" style="7" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="11" style="7" customWidth="1"/>
     <col min="6" max="6" width="9.7109375" style="21" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.140625" style="6"/>
     <col min="10" max="10" width="11.85546875" bestFit="1" customWidth="1"/>
@@ -22168,7 +22167,7 @@
         <v>3509</v>
       </c>
       <c r="E6" s="71">
-        <v>121</v>
+        <v>101</v>
       </c>
       <c r="F6" s="70">
         <v>182</v>
@@ -22260,7 +22259,7 @@
         <v>3513</v>
       </c>
       <c r="E10" s="71">
-        <v>288</v>
+        <v>278</v>
       </c>
       <c r="F10" s="70">
         <v>225</v>
@@ -31945,7 +31944,7 @@
         <v>2306</v>
       </c>
       <c r="E36" s="19">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F36" s="17">
         <v>418</v>
@@ -32111,7 +32110,7 @@
         <v>1331</v>
       </c>
       <c r="E44" s="19">
-        <v>331</v>
+        <v>375</v>
       </c>
       <c r="F44" s="17">
         <v>247</v>
@@ -32132,7 +32131,7 @@
         <v>1331</v>
       </c>
       <c r="E45" s="19">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F45" s="17">
         <v>676</v>
@@ -32172,7 +32171,7 @@
       </c>
       <c r="D47" s="17"/>
       <c r="E47" s="19">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F47" s="17"/>
       <c r="G47" s="32"/>
@@ -32522,7 +32521,7 @@
         <v>2865</v>
       </c>
       <c r="E64" s="84">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="F64" s="32">
         <v>251</v>
@@ -33387,7 +33386,7 @@
         <v>2450</v>
       </c>
       <c r="E15">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F15">
         <v>935</v>
@@ -35991,7 +35990,7 @@
       </c>
       <c r="D7" s="26"/>
       <c r="E7" s="9">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F7" s="9"/>
     </row>
@@ -36009,7 +36008,7 @@
         <v>2378</v>
       </c>
       <c r="E8" s="9">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F8" s="9"/>
     </row>
@@ -43096,7 +43095,7 @@
       <c r="C100" s="33"/>
       <c r="D100" s="38"/>
       <c r="E100" s="35">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F100" s="33" t="s">
         <v>2650</v>
@@ -47950,7 +47949,7 @@
       </c>
       <c r="D183" s="33"/>
       <c r="E183" s="35">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F183" s="33"/>
     </row>
@@ -48236,7 +48235,7 @@
       </c>
       <c r="D200" s="33"/>
       <c r="E200" s="35">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F200" s="33"/>
     </row>
@@ -49309,7 +49308,7 @@
         <v>399</v>
       </c>
       <c r="E263" s="35">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F263" s="33">
         <v>645</v>
@@ -49711,7 +49710,7 @@
       </c>
       <c r="D288" s="33"/>
       <c r="E288" s="35">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="F288" s="33"/>
     </row>
@@ -49835,7 +49834,7 @@
       </c>
       <c r="D295" s="33"/>
       <c r="E295" s="35">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F295" s="33">
         <v>696</v>
@@ -50198,7 +50197,7 @@
       </c>
       <c r="D316" s="33"/>
       <c r="E316" s="35">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F316" s="33">
         <v>865</v>
@@ -50378,7 +50377,7 @@
         <v>3323</v>
       </c>
       <c r="E326" s="35">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F326" s="33" t="s">
         <v>2820</v>
@@ -53624,7 +53623,7 @@
         <v>2703</v>
       </c>
       <c r="E127" s="56">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="F127" s="35">
         <v>772</v>
@@ -54524,7 +54523,7 @@
         <v>2703</v>
       </c>
       <c r="E175" s="56">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F175" s="56">
         <v>2310</v>
@@ -57174,7 +57173,7 @@
       </c>
       <c r="D4" s="33"/>
       <c r="E4" s="33">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="F4" s="35">
         <v>146</v>
@@ -57281,7 +57280,7 @@
       </c>
       <c r="D10" s="33"/>
       <c r="E10" s="33">
-        <v>829</v>
+        <v>798</v>
       </c>
       <c r="F10" s="35">
         <v>193</v>
@@ -57448,7 +57447,7 @@
       </c>
       <c r="D19" s="33"/>
       <c r="E19" s="33">
-        <v>51</v>
+        <v>91</v>
       </c>
       <c r="F19" s="35" t="s">
         <v>2788</v>
@@ -57688,7 +57687,7 @@
         <v>3358</v>
       </c>
       <c r="E32" s="60">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="F32" s="33">
         <v>424</v>
@@ -58160,7 +58159,7 @@
         <v>3397</v>
       </c>
       <c r="E58" s="42">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F58" s="35">
         <v>408</v>
@@ -58328,7 +58327,7 @@
       </c>
       <c r="D68" s="33"/>
       <c r="E68" s="33">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="F68" s="35">
         <v>208</v>
@@ -58506,7 +58505,7 @@
       </c>
       <c r="D78" s="33"/>
       <c r="E78" s="33">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="F78" s="35">
         <v>253</v>
@@ -58758,7 +58757,7 @@
       </c>
       <c r="D92" s="33"/>
       <c r="E92" s="33">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F92" s="35">
         <v>1325</v>
@@ -58963,7 +58962,7 @@
       </c>
       <c r="D103" s="33"/>
       <c r="E103" s="33">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F103" s="35">
         <v>335</v>
@@ -59151,7 +59150,7 @@
       </c>
       <c r="D113" s="33"/>
       <c r="E113" s="33">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F113" s="35">
         <v>746</v>
@@ -59573,7 +59572,7 @@
       </c>
       <c r="D136" s="33"/>
       <c r="E136" s="33">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="F136" s="33">
         <v>1045</v>
@@ -60003,7 +60002,7 @@
         <v>1858</v>
       </c>
       <c r="E160" s="33">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="F160" s="35">
         <v>234</v>
@@ -60043,7 +60042,7 @@
         <v>3406</v>
       </c>
       <c r="E162" s="33">
-        <v>41</v>
+        <v>59</v>
       </c>
       <c r="F162" s="35">
         <v>638</v>
@@ -60063,7 +60062,7 @@
         <v>3408</v>
       </c>
       <c r="E163" s="33">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="F163" s="35">
         <v>686</v>
@@ -60083,7 +60082,7 @@
         <v>3409</v>
       </c>
       <c r="E164" s="60">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="F164" s="33">
         <v>868</v>
@@ -60123,7 +60122,7 @@
         <v>3411</v>
       </c>
       <c r="E166" s="33">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F166" s="35" t="s">
         <v>2848</v>
@@ -60183,7 +60182,7 @@
         <v>3415</v>
       </c>
       <c r="E169" s="33">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F169" s="35">
         <v>1454</v>
@@ -60453,7 +60452,7 @@
         <v>290</v>
       </c>
       <c r="E183" s="33">
-        <v>37</v>
+        <v>117</v>
       </c>
       <c r="F183" s="35">
         <v>170</v>
@@ -60671,7 +60670,7 @@
         <v>2799</v>
       </c>
       <c r="E194" s="42">
-        <v>22</v>
+        <v>247</v>
       </c>
       <c r="F194" s="35">
         <v>170</v>
@@ -60691,7 +60690,7 @@
         <v>3436</v>
       </c>
       <c r="E195" s="42">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F195" s="35" t="s">
         <v>3005</v>
@@ -61117,7 +61116,7 @@
         <v>3451</v>
       </c>
       <c r="E217" s="33">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F217" s="33">
         <v>330</v>
@@ -61137,7 +61136,7 @@
         <v>3452</v>
       </c>
       <c r="E218" s="33">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="F218" s="33" t="s">
         <v>2940</v>
@@ -61417,7 +61416,7 @@
         <v>3464</v>
       </c>
       <c r="E232" s="33">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F232" s="35">
         <v>1026</v>
@@ -61557,7 +61556,7 @@
         <v>3471</v>
       </c>
       <c r="E239" s="33">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="F239" s="35">
         <v>494</v>
@@ -61617,7 +61616,7 @@
         <v>3474</v>
       </c>
       <c r="E242" s="33">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="F242" s="35">
         <v>258</v>
@@ -61775,7 +61774,7 @@
       </c>
       <c r="D250" s="33"/>
       <c r="E250" s="33">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F250" s="35" t="s">
         <v>2943</v>
@@ -61815,7 +61814,7 @@
         <v>2884</v>
       </c>
       <c r="E252" s="33">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="F252" s="35">
         <v>567</v>
@@ -61953,7 +61952,7 @@
         <v>2988</v>
       </c>
       <c r="E259" s="33">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="F259" s="35">
         <v>505</v>
@@ -62111,7 +62110,7 @@
         <v>3575</v>
       </c>
       <c r="E267" s="33">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="F267" s="35">
         <v>536</v>
@@ -63839,7 +63838,7 @@
       <c r="C65" s="4"/>
       <c r="D65" s="4"/>
       <c r="E65" s="62">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F65" s="4">
         <v>4394</v>
@@ -65148,7 +65147,7 @@
       </c>
       <c r="D9" s="33"/>
       <c r="E9" s="35">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="F9" s="33" t="s">
         <v>2814</v>
@@ -65947,7 +65946,7 @@
         <v>2294</v>
       </c>
       <c r="E54" s="35">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F54" s="33">
         <v>5355</v>

</xml_diff>

<commit_message>
feat: Implement catalogue fetching and display functionality with new components and styles
</commit_message>
<xml_diff>
--- a/backend/public/BOSCH_STOCK1.xlsx
+++ b/backend/public/BOSCH_STOCK1.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="12240" windowHeight="9240" tabRatio="730" firstSheet="3" activeTab="5"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="12240" windowHeight="9240" tabRatio="730" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="ELEMENT" sheetId="1" r:id="rId1"/>
@@ -12864,7 +12864,7 @@
       </c>
       <c r="D32" s="17"/>
       <c r="E32" s="19">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
@@ -14276,7 +14276,7 @@
       </c>
       <c r="D100" s="17"/>
       <c r="E100" s="19">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F100" s="17" t="s">
         <v>2650</v>
@@ -14891,7 +14891,7 @@
       </c>
       <c r="D129" s="17"/>
       <c r="E129" s="19">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F129" s="17"/>
       <c r="G129" s="17"/>
@@ -15181,7 +15181,7 @@
       </c>
       <c r="D143" s="17"/>
       <c r="E143" s="19">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F143" s="17"/>
       <c r="G143" s="17"/>
@@ -15486,7 +15486,7 @@
       </c>
       <c r="D158" s="17"/>
       <c r="E158" s="19">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F158" s="17"/>
       <c r="G158" s="17"/>
@@ -16230,7 +16230,7 @@
         <v>2703</v>
       </c>
       <c r="E6" s="75">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F6" s="74">
         <v>2322</v>
@@ -18852,7 +18852,7 @@
         <v>822</v>
       </c>
       <c r="E142" s="75">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="F142" s="74">
         <v>746</v>
@@ -19058,7 +19058,7 @@
         <v>1396</v>
       </c>
       <c r="E152" s="75">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F152" s="74">
         <v>969</v>
@@ -19892,7 +19892,7 @@
       <c r="C193" s="74"/>
       <c r="D193" s="74"/>
       <c r="E193" s="75">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F193" s="74">
         <v>2405</v>
@@ -20590,7 +20590,7 @@
         <v>2441</v>
       </c>
       <c r="E228" s="75">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F228" s="74">
         <v>14552</v>
@@ -22167,7 +22167,7 @@
         <v>3509</v>
       </c>
       <c r="E6" s="71">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="F6" s="70">
         <v>182</v>
@@ -22331,7 +22331,7 @@
         <v>3516</v>
       </c>
       <c r="E13" s="71">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="F13" s="70">
         <v>288</v>
@@ -31505,7 +31505,7 @@
         <v>1303</v>
       </c>
       <c r="E15" s="19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F15" s="17">
         <v>6968</v>
@@ -31818,7 +31818,7 @@
         <v>2372</v>
       </c>
       <c r="E30" s="19">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="F30" s="17">
         <v>1709</v>
@@ -32110,7 +32110,7 @@
         <v>1331</v>
       </c>
       <c r="E44" s="19">
-        <v>375</v>
+        <v>361</v>
       </c>
       <c r="F44" s="17">
         <v>247</v>
@@ -33206,7 +33206,7 @@
         <v>2246</v>
       </c>
       <c r="E6">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F6">
         <v>815</v>
@@ -36008,7 +36008,7 @@
         <v>2378</v>
       </c>
       <c r="E8" s="9">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F8" s="9"/>
     </row>
@@ -36966,7 +36966,7 @@
         <v>693</v>
       </c>
       <c r="E61" s="10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F61" s="9"/>
     </row>
@@ -37038,7 +37038,7 @@
         <v>769</v>
       </c>
       <c r="E65" s="10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F65" s="9"/>
     </row>
@@ -40138,7 +40138,7 @@
         <v>1542</v>
       </c>
       <c r="E217" s="10">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F217" s="9"/>
       <c r="G217" t="s">
@@ -42656,7 +42656,7 @@
       <c r="C74" s="33"/>
       <c r="D74" s="38"/>
       <c r="E74" s="35">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F74" s="33"/>
       <c r="H74" t="s">
@@ -42960,7 +42960,7 @@
       <c r="C92" s="33"/>
       <c r="D92" s="38"/>
       <c r="E92" s="35">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F92" s="33"/>
       <c r="H92" t="s">
@@ -42977,7 +42977,7 @@
       <c r="C93" s="33"/>
       <c r="D93" s="38"/>
       <c r="E93" s="35">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F93" s="33" t="s">
         <v>2596</v>
@@ -43095,7 +43095,7 @@
       <c r="C100" s="33"/>
       <c r="D100" s="38"/>
       <c r="E100" s="35">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F100" s="33" t="s">
         <v>2650</v>
@@ -45683,7 +45683,7 @@
       </c>
       <c r="D43" s="33"/>
       <c r="E43" s="35">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F43" s="33">
         <v>154</v>
@@ -45797,7 +45797,7 @@
       </c>
       <c r="D50" s="33"/>
       <c r="E50" s="35">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F50" s="33"/>
     </row>
@@ -47117,7 +47117,7 @@
       </c>
       <c r="D132" s="33"/>
       <c r="E132" s="35">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F132" s="33">
         <v>247</v>
@@ -49710,7 +49710,7 @@
       </c>
       <c r="D288" s="33"/>
       <c r="E288" s="35">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="F288" s="33"/>
     </row>
@@ -49816,7 +49816,7 @@
       </c>
       <c r="D294" s="33"/>
       <c r="E294" s="35">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="F294" s="33">
         <v>696</v>
@@ -52384,7 +52384,7 @@
         <v>2697</v>
       </c>
       <c r="E57" s="56">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F57" s="35">
         <v>2075</v>
@@ -52520,7 +52520,7 @@
         <v>2703</v>
       </c>
       <c r="E65" s="56">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F65" s="35" t="s">
         <v>2764</v>
@@ -53696,7 +53696,7 @@
         <v>2698</v>
       </c>
       <c r="E131" s="56">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F131" s="35" t="s">
         <v>3127</v>
@@ -53734,7 +53734,7 @@
         <v>2706</v>
       </c>
       <c r="E133" s="56">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F133" s="35" t="s">
         <v>3584</v>
@@ -53797,7 +53797,7 @@
         <v>518894</v>
       </c>
       <c r="E136" s="56">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="F136" s="35" t="s">
         <v>3582</v>
@@ -54699,7 +54699,7 @@
         <v>2709</v>
       </c>
       <c r="E184" s="56">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F184" s="35">
         <v>1739</v>
@@ -54832,7 +54832,7 @@
         <v>2703</v>
       </c>
       <c r="E191" s="56">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F191" s="35">
         <v>1106</v>
@@ -57280,7 +57280,7 @@
       </c>
       <c r="D10" s="33"/>
       <c r="E10" s="33">
-        <v>798</v>
+        <v>768</v>
       </c>
       <c r="F10" s="35">
         <v>193</v>
@@ -57298,7 +57298,7 @@
       </c>
       <c r="D11" s="33"/>
       <c r="E11" s="33">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F11" s="35">
         <v>184</v>
@@ -57316,7 +57316,7 @@
       </c>
       <c r="D12" s="33"/>
       <c r="E12" s="33">
-        <v>724</v>
+        <v>709</v>
       </c>
       <c r="F12" s="35">
         <v>184</v>
@@ -57393,7 +57393,7 @@
       </c>
       <c r="D16" s="33"/>
       <c r="E16" s="33">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="F16" s="35">
         <v>400</v>
@@ -57411,7 +57411,7 @@
       </c>
       <c r="D17" s="33"/>
       <c r="E17" s="33">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="F17" s="35">
         <v>396</v>
@@ -57627,7 +57627,7 @@
         <v>3355</v>
       </c>
       <c r="E29" s="60">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="F29" s="33">
         <v>379</v>
@@ -57667,7 +57667,7 @@
         <v>3357</v>
       </c>
       <c r="E31" s="60">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F31" s="35">
         <v>268</v>
@@ -57687,7 +57687,7 @@
         <v>3358</v>
       </c>
       <c r="E32" s="60">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="F32" s="33">
         <v>424</v>
@@ -58139,7 +58139,7 @@
       </c>
       <c r="D57" s="33"/>
       <c r="E57" s="33">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F57" s="35">
         <v>260</v>
@@ -59328,7 +59328,7 @@
       </c>
       <c r="D123" s="33"/>
       <c r="E123" s="33">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F123" s="35">
         <v>197</v>
@@ -60062,7 +60062,7 @@
         <v>3408</v>
       </c>
       <c r="E163" s="33">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="F163" s="35">
         <v>686</v>
@@ -60162,7 +60162,7 @@
         <v>3413</v>
       </c>
       <c r="E168" s="33">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F168" s="35">
         <v>451</v>
@@ -60322,7 +60322,7 @@
         <v>3425</v>
       </c>
       <c r="E176" s="33">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="F176" s="35">
         <v>282</v>
@@ -60472,7 +60472,7 @@
         <v>318</v>
       </c>
       <c r="E184" s="33">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="F184" s="35">
         <v>186</v>
@@ -60592,7 +60592,7 @@
         <v>3433</v>
       </c>
       <c r="E190" s="33">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="F190" s="33" t="s">
         <v>3022</v>
@@ -60906,7 +60906,7 @@
         <v>3587</v>
       </c>
       <c r="E206" s="33">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F206" s="35">
         <v>300</v>
@@ -61116,7 +61116,7 @@
         <v>3451</v>
       </c>
       <c r="E217" s="33">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F217" s="33">
         <v>330</v>
@@ -61156,7 +61156,7 @@
         <v>2392</v>
       </c>
       <c r="E219" s="33">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F219" s="33">
         <v>244</v>
@@ -61436,7 +61436,7 @@
         <v>3465</v>
       </c>
       <c r="E233" s="33">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="F233" s="35">
         <v>353</v>
@@ -62273,7 +62273,7 @@
         <v>3484</v>
       </c>
       <c r="E276" s="33">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F276" s="33">
         <v>239</v>
@@ -63742,7 +63742,7 @@
         <v>401</v>
       </c>
       <c r="E60" s="62">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F60" s="4"/>
       <c r="G60" s="4"/>
@@ -65497,7 +65497,7 @@
       </c>
       <c r="D29" s="33"/>
       <c r="E29" s="35">
-        <v>330</v>
+        <v>310</v>
       </c>
       <c r="F29" s="33">
         <v>21</v>

</xml_diff>

<commit_message>
Update stock files: replace BOSCH_STOCK1.xlsx and LUCAS_STOCK.xlsx with new versions
</commit_message>
<xml_diff>
--- a/backend/public/BOSCH_STOCK1.xlsx
+++ b/backend/public/BOSCH_STOCK1.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="12240" windowHeight="9240" tabRatio="730"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="12240" windowHeight="9240" tabRatio="730" firstSheet="10" activeTab="13"/>
   </bookViews>
   <sheets>
     <sheet name="ELEMENT" sheetId="1" r:id="rId1"/>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5811" uniqueCount="3599">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5810" uniqueCount="3598">
   <si>
     <t>0 433 175 443</t>
   </si>
@@ -10860,9 +10860,6 @@
   </si>
   <si>
     <t>285/262</t>
-  </si>
-  <si>
-    <t>2102/1937</t>
   </si>
   <si>
     <t>8125/7490</t>
@@ -14923,7 +14920,7 @@
       </c>
       <c r="D129" s="17"/>
       <c r="E129" s="19">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F129" s="17"/>
       <c r="G129" s="17"/>
@@ -15644,7 +15641,7 @@
     <row r="165" spans="1:10" ht="15.75">
       <c r="A165" s="17"/>
       <c r="B165" s="17" t="s">
-        <v>3589</v>
+        <v>3588</v>
       </c>
       <c r="C165" s="18" t="s">
         <v>3145</v>
@@ -16484,7 +16481,7 @@
         <v>70</v>
       </c>
       <c r="F16" s="74" t="s">
-        <v>3593</v>
+        <v>3592</v>
       </c>
       <c r="G16" s="74"/>
       <c r="H16" s="74"/>
@@ -19861,10 +19858,10 @@
       </c>
       <c r="D189" s="74"/>
       <c r="E189" s="75">
-        <v>5</v>
-      </c>
-      <c r="F189" s="74" t="s">
-        <v>3570</v>
+        <v>7</v>
+      </c>
+      <c r="F189" s="74">
+        <v>2275</v>
       </c>
       <c r="G189" s="74"/>
       <c r="H189" s="74"/>
@@ -20458,7 +20455,7 @@
     <row r="220" spans="1:8" ht="21">
       <c r="A220" s="74"/>
       <c r="B220" s="74" t="s">
-        <v>3575</v>
+        <v>3574</v>
       </c>
       <c r="C220" s="74" t="s">
         <v>598</v>
@@ -20576,7 +20573,7 @@
         <v>2</v>
       </c>
       <c r="F225" s="74" t="s">
-        <v>3585</v>
+        <v>3584</v>
       </c>
       <c r="G225" s="74"/>
       <c r="H225" s="74"/>
@@ -20620,7 +20617,7 @@
         <v>1</v>
       </c>
       <c r="F227" s="74" t="s">
-        <v>3592</v>
+        <v>3591</v>
       </c>
       <c r="G227" s="74"/>
       <c r="H227" s="74"/>
@@ -21050,7 +21047,7 @@
         <v>0</v>
       </c>
       <c r="F247" s="74" t="s">
-        <v>3571</v>
+        <v>3570</v>
       </c>
       <c r="G247" s="74"/>
       <c r="H247" s="74"/>
@@ -22037,7 +22034,7 @@
     </row>
     <row r="294" spans="1:8" ht="21">
       <c r="B294" s="90" t="s">
-        <v>3590</v>
+        <v>3589</v>
       </c>
       <c r="C294" s="74" t="s">
         <v>843</v>
@@ -22502,7 +22499,7 @@
         <v>2604</v>
       </c>
       <c r="E18" s="71">
-        <v>65</v>
+        <v>15</v>
       </c>
       <c r="F18" s="69">
         <v>392</v>
@@ -22568,7 +22565,7 @@
         <v>2227</v>
       </c>
       <c r="E21" s="71">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F21" s="69">
         <v>482</v>
@@ -31406,7 +31403,7 @@
         <v>1292</v>
       </c>
       <c r="E7" s="19">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F7" s="17">
         <v>3385</v>
@@ -32011,7 +32008,7 @@
         <v>2303</v>
       </c>
       <c r="E36" s="19">
-        <v>74</v>
+        <v>104</v>
       </c>
       <c r="F36" s="17">
         <v>418</v>
@@ -32571,7 +32568,7 @@
         <v>3080</v>
       </c>
       <c r="H63" s="8" t="s">
-        <v>3596</v>
+        <v>3595</v>
       </c>
     </row>
     <row r="64" spans="1:8" ht="15.75">
@@ -33377,7 +33374,7 @@
         <v>0</v>
       </c>
       <c r="F11" t="s">
-        <v>3583</v>
+        <v>3582</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -33854,10 +33851,10 @@
         <v>836</v>
       </c>
       <c r="E35">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F35" t="s">
-        <v>3598</v>
+        <v>3597</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -33974,7 +33971,7 @@
         <v>1747</v>
       </c>
       <c r="E41">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F41">
         <v>953</v>
@@ -34317,7 +34314,7 @@
         <v>4</v>
       </c>
       <c r="F58" t="s">
-        <v>3597</v>
+        <v>3596</v>
       </c>
     </row>
     <row r="59" spans="1:6">
@@ -35049,7 +35046,7 @@
     </row>
     <row r="98" spans="1:6">
       <c r="B98" s="6" t="s">
-        <v>3573</v>
+        <v>3572</v>
       </c>
       <c r="C98" t="s">
         <v>3546</v>
@@ -40198,7 +40195,7 @@
         <v>1542</v>
       </c>
       <c r="E217" s="10">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F217" s="9"/>
       <c r="G217" t="s">
@@ -41470,7 +41467,7 @@
       </c>
       <c r="D6" s="38"/>
       <c r="E6" s="35">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F6" s="33"/>
       <c r="H6" t="s">
@@ -42716,7 +42713,7 @@
       <c r="C74" s="33"/>
       <c r="D74" s="38"/>
       <c r="E74" s="35">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F74" s="33"/>
       <c r="H74" t="s">
@@ -45857,7 +45854,7 @@
       </c>
       <c r="D50" s="33"/>
       <c r="E50" s="35">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F50" s="33"/>
     </row>
@@ -49256,7 +49253,7 @@
       </c>
       <c r="D257" s="33"/>
       <c r="E257" s="35">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F257" s="33">
         <v>137</v>
@@ -49306,7 +49303,7 @@
         <v>1169</v>
       </c>
       <c r="C260" s="33" t="s">
-        <v>3595</v>
+        <v>3594</v>
       </c>
       <c r="D260" s="33" t="s">
         <v>1170</v>
@@ -49448,7 +49445,7 @@
       <c r="C268" s="33"/>
       <c r="D268" s="33"/>
       <c r="E268" s="35">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F268" s="33"/>
     </row>
@@ -49770,7 +49767,7 @@
       </c>
       <c r="D288" s="33"/>
       <c r="E288" s="35">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="F288" s="33"/>
     </row>
@@ -49876,7 +49873,7 @@
       </c>
       <c r="D294" s="33"/>
       <c r="E294" s="35">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F294" s="33">
         <v>696</v>
@@ -50257,7 +50254,7 @@
       </c>
       <c r="D316" s="33"/>
       <c r="E316" s="35">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F316" s="33">
         <v>865</v>
@@ -50362,7 +50359,7 @@
         <v>1207</v>
       </c>
       <c r="D322" s="33" t="s">
-        <v>3580</v>
+        <v>3579</v>
       </c>
       <c r="E322" s="35">
         <v>40</v>
@@ -50382,7 +50379,7 @@
         <v>1207</v>
       </c>
       <c r="D323" s="33" t="s">
-        <v>3581</v>
+        <v>3580</v>
       </c>
       <c r="E323" s="35">
         <v>36</v>
@@ -50431,7 +50428,7 @@
         <v>3281</v>
       </c>
       <c r="C326" s="33" t="s">
-        <v>3582</v>
+        <v>3581</v>
       </c>
       <c r="D326" s="33" t="s">
         <v>3314</v>
@@ -50506,7 +50503,7 @@
         <v>329</v>
       </c>
       <c r="B330" s="33" t="s">
-        <v>3579</v>
+        <v>3578</v>
       </c>
       <c r="C330" s="33" t="s">
         <v>3315</v>
@@ -51341,10 +51338,10 @@
     </row>
     <row r="377" spans="1:6">
       <c r="B377" s="34" t="s">
+        <v>3585</v>
+      </c>
+      <c r="C377" s="89" t="s">
         <v>3586</v>
-      </c>
-      <c r="C377" s="89" t="s">
-        <v>3587</v>
       </c>
       <c r="E377" s="1">
         <v>5</v>
@@ -53159,7 +53156,7 @@
         <v>4</v>
       </c>
       <c r="F96" s="35" t="s">
-        <v>3588</v>
+        <v>3587</v>
       </c>
     </row>
     <row r="97" spans="1:7">
@@ -53813,7 +53810,7 @@
         <v>8</v>
       </c>
       <c r="F133" s="35" t="s">
-        <v>3574</v>
+        <v>3573</v>
       </c>
     </row>
     <row r="134" spans="1:7">
@@ -53873,10 +53870,10 @@
         <v>518894</v>
       </c>
       <c r="E136" s="56">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F136" s="35" t="s">
-        <v>3572</v>
+        <v>3571</v>
       </c>
     </row>
     <row r="137" spans="1:7">
@@ -54242,7 +54239,7 @@
         <v>2700</v>
       </c>
       <c r="E156" s="56">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F156" s="35">
         <v>1092</v>
@@ -57331,7 +57328,7 @@
     <row r="9" spans="1:10">
       <c r="A9" s="33"/>
       <c r="B9" s="33" t="s">
-        <v>3578</v>
+        <v>3577</v>
       </c>
       <c r="C9" s="33" t="s">
         <v>1210</v>
@@ -57356,7 +57353,7 @@
       </c>
       <c r="D10" s="33"/>
       <c r="E10" s="33">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="F10" s="35">
         <v>193</v>
@@ -58147,7 +58144,7 @@
       </c>
       <c r="D53" s="33"/>
       <c r="E53" s="33">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F53" s="35">
         <v>276</v>
@@ -58183,7 +58180,7 @@
       </c>
       <c r="D55" s="33"/>
       <c r="E55" s="33">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="F55" s="35">
         <v>260</v>
@@ -59478,7 +59475,7 @@
     <row r="127" spans="1:8">
       <c r="A127" s="33"/>
       <c r="B127" s="33" t="s">
-        <v>3584</v>
+        <v>3583</v>
       </c>
       <c r="C127" s="33" t="s">
         <v>1276</v>
@@ -60675,7 +60672,7 @@
         <v>39</v>
       </c>
       <c r="F190" s="35" t="s">
-        <v>3591</v>
+        <v>3590</v>
       </c>
     </row>
     <row r="191" spans="1:6">
@@ -60957,13 +60954,13 @@
     <row r="205" spans="1:6">
       <c r="A205" s="33"/>
       <c r="B205" s="33" t="s">
-        <v>3576</v>
+        <v>3575</v>
       </c>
       <c r="C205" s="33" t="s">
         <v>3365</v>
       </c>
       <c r="D205" s="33" t="s">
-        <v>3577</v>
+        <v>3576</v>
       </c>
       <c r="E205" s="33">
         <v>6</v>
@@ -61476,7 +61473,7 @@
         <v>3455</v>
       </c>
       <c r="E231" s="33">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F231" s="35">
         <v>1026</v>
@@ -62450,7 +62447,7 @@
         <v>2377</v>
       </c>
       <c r="D281" s="33" t="s">
-        <v>3594</v>
+        <v>3593</v>
       </c>
       <c r="E281" s="33">
         <v>27</v>
@@ -65506,7 +65503,7 @@
       </c>
       <c r="D26" s="33"/>
       <c r="E26" s="35">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="F26" s="33">
         <v>18</v>
@@ -65556,7 +65553,7 @@
       </c>
       <c r="D29" s="33"/>
       <c r="E29" s="35">
-        <v>110</v>
+        <v>210</v>
       </c>
       <c r="F29" s="33">
         <v>21</v>

</xml_diff>